<commit_message>
some random changes & improvements
</commit_message>
<xml_diff>
--- a/Caddie POC - Result Validation.xlsx
+++ b/Caddie POC - Result Validation.xlsx
@@ -13727,7 +13727,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -13844,10 +13844,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14266,7 +14263,7 @@
       <c r="B2" s="8">
         <v>1</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="8" t="s">
         <v>47</v>
       </c>
       <c r="D2" s="25"/>
@@ -14291,7 +14288,7 @@
       <c r="B3" s="8">
         <v>2</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="44" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="9"/>
@@ -14310,7 +14307,7 @@
       <c r="B4" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="44" t="s">
         <v>55</v>
       </c>
       <c r="D4" s="9"/>
@@ -14327,7 +14324,7 @@
       <c r="B5" s="8">
         <v>3</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="8" t="s">
         <v>56</v>
       </c>
       <c r="D5" s="9" t="e">
@@ -14357,7 +14354,7 @@
       <c r="B6" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="8" t="s">
         <v>63</v>
       </c>
       <c r="D6" s="9" t="e">
@@ -14385,7 +14382,7 @@
       <c r="B7" s="8">
         <v>5</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="8" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="9" t="e">
@@ -14410,7 +14407,7 @@
       <c r="B8" s="8">
         <v>6</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="8" t="s">
         <v>71</v>
       </c>
       <c r="D8" s="9" t="e">
@@ -14437,7 +14434,7 @@
       <c r="B9" s="8">
         <v>7</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="8" t="s">
         <v>75</v>
       </c>
       <c r="D9" s="9" t="s">
@@ -14456,7 +14453,7 @@
       <c r="B10" s="8">
         <v>8</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -14483,7 +14480,7 @@
       <c r="B11" s="8">
         <v>11</v>
       </c>
-      <c r="C11" s="44" t="s">
+      <c r="C11" s="8" t="s">
         <v>82</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -14510,7 +14507,7 @@
       <c r="B12" s="8">
         <v>13</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="8" t="s">
         <v>87</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -14535,7 +14532,7 @@
       <c r="B13" s="8">
         <v>17</v>
       </c>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="8" t="s">
         <v>91</v>
       </c>
       <c r="D13" s="6" t="s">
@@ -14562,7 +14559,7 @@
       <c r="B14" s="8">
         <v>18</v>
       </c>
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="8" t="s">
         <v>96</v>
       </c>
       <c r="D14" s="6" t="s">
@@ -14587,7 +14584,7 @@
       <c r="B15" s="8">
         <v>21</v>
       </c>
-      <c r="C15" s="44" t="s">
+      <c r="C15" s="8" t="s">
         <v>100</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -14606,7 +14603,7 @@
       <c r="B16" s="8">
         <v>25</v>
       </c>
-      <c r="C16" s="44" t="s">
+      <c r="C16" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -14635,7 +14632,7 @@
       <c r="B17" s="8">
         <v>26</v>
       </c>
-      <c r="C17" s="44" t="s">
+      <c r="C17" s="8" t="s">
         <v>108</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -14660,7 +14657,7 @@
       <c r="B18" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -14687,7 +14684,7 @@
       <c r="B19" s="8">
         <v>27</v>
       </c>
-      <c r="C19" s="44" t="s">
+      <c r="C19" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D19" s="6" t="s">
@@ -14719,7 +14716,7 @@
       <c r="B20" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="C20" s="8" t="s">
         <v>126</v>
       </c>
       <c r="D20" s="6" t="s">
@@ -14746,7 +14743,7 @@
       <c r="B21" s="8">
         <v>28</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="C21" s="8" t="s">
         <v>131</v>
       </c>
       <c r="D21" s="6" t="s">
@@ -14775,7 +14772,7 @@
       <c r="B22" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C22" s="44" t="s">
+      <c r="C22" s="8" t="s">
         <v>138</v>
       </c>
       <c r="D22" s="6" t="s">
@@ -14802,7 +14799,7 @@
       <c r="B23" s="8">
         <v>29</v>
       </c>
-      <c r="C23" s="44" t="s">
+      <c r="C23" s="8" t="s">
         <v>143</v>
       </c>
       <c r="D23" s="6" t="s">
@@ -14829,7 +14826,7 @@
       <c r="B24" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C24" s="44" t="s">
+      <c r="C24" s="8" t="s">
         <v>149</v>
       </c>
       <c r="D24" s="14" t="s">
@@ -14856,7 +14853,7 @@
       <c r="B25" s="8">
         <v>30</v>
       </c>
-      <c r="C25" s="44" t="s">
+      <c r="C25" s="8" t="s">
         <v>153</v>
       </c>
       <c r="D25" s="26" t="s">
@@ -14877,7 +14874,7 @@
       <c r="B26" s="8">
         <v>31</v>
       </c>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D26" s="14" t="s">
@@ -14906,7 +14903,7 @@
       <c r="B27" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="44" t="s">
+      <c r="C27" s="8" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="14" t="s">
@@ -14935,7 +14932,7 @@
       <c r="B28" s="8">
         <v>32</v>
       </c>
-      <c r="C28" s="44" t="s">
+      <c r="C28" s="8" t="s">
         <v>26</v>
       </c>
       <c r="D28" s="14" t="s">
@@ -14964,7 +14961,7 @@
       <c r="B29" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="44" t="s">
+      <c r="C29" s="8" t="s">
         <v>31</v>
       </c>
       <c r="D29" s="15" t="s">
@@ -14993,7 +14990,7 @@
       <c r="B30" s="8">
         <v>34</v>
       </c>
-      <c r="C30" s="44" t="s">
+      <c r="C30" s="8" t="s">
         <v>173</v>
       </c>
       <c r="D30" s="15" t="s">
@@ -15022,7 +15019,7 @@
       <c r="B31" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C31" s="44" t="s">
+      <c r="C31" s="8" t="s">
         <v>179</v>
       </c>
       <c r="D31" s="15" t="s">
@@ -15051,7 +15048,7 @@
       <c r="B32" s="8">
         <v>38</v>
       </c>
-      <c r="C32" s="44" t="s">
+      <c r="C32" s="8" t="s">
         <v>184</v>
       </c>
       <c r="D32" s="15" t="s">
@@ -15080,7 +15077,7 @@
       <c r="B33" s="8">
         <v>43</v>
       </c>
-      <c r="C33" s="44" t="s">
+      <c r="C33" s="8" t="s">
         <v>35</v>
       </c>
       <c r="D33" s="15" t="s">
@@ -15109,7 +15106,7 @@
       <c r="B34" s="8">
         <v>44</v>
       </c>
-      <c r="C34" s="44" t="s">
+      <c r="C34" s="8" t="s">
         <v>193</v>
       </c>
       <c r="D34" s="15" t="s">
@@ -15138,7 +15135,7 @@
       <c r="B35" s="8">
         <v>46</v>
       </c>
-      <c r="C35" s="44" t="s">
+      <c r="C35" s="8" t="s">
         <v>39</v>
       </c>
       <c r="D35" s="15" t="s">
@@ -15167,7 +15164,7 @@
       <c r="B36" s="8">
         <v>47</v>
       </c>
-      <c r="C36" s="44" t="s">
+      <c r="C36" s="8" t="s">
         <v>204</v>
       </c>
       <c r="D36" s="15" t="s">
@@ -15196,7 +15193,7 @@
       <c r="B37" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="C37" s="44" t="s">
+      <c r="C37" s="8" t="s">
         <v>211</v>
       </c>
       <c r="D37" s="15" t="s">
@@ -15223,7 +15220,7 @@
       <c r="B38" s="8">
         <v>48</v>
       </c>
-      <c r="C38" s="44" t="s">
+      <c r="C38" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D38" s="15" t="s">
@@ -15252,7 +15249,7 @@
       <c r="B39" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="C39" s="44" t="s">
+      <c r="C39" s="8" t="s">
         <v>222</v>
       </c>
       <c r="D39" s="15" t="s">
@@ -15281,7 +15278,7 @@
       <c r="B40" s="8">
         <v>50</v>
       </c>
-      <c r="C40" s="44" t="s">
+      <c r="C40" s="8" t="s">
         <v>227</v>
       </c>
       <c r="D40" s="14" t="s">
@@ -15310,7 +15307,7 @@
       <c r="B41" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C41" s="44" t="s">
+      <c r="C41" s="8" t="s">
         <v>234</v>
       </c>
       <c r="D41" s="15" t="s">
@@ -15339,7 +15336,7 @@
       <c r="B42" s="8">
         <v>51</v>
       </c>
-      <c r="C42" s="44" t="s">
+      <c r="C42" s="8" t="s">
         <v>239</v>
       </c>
       <c r="D42" s="15" t="s">
@@ -15369,7 +15366,7 @@
       <c r="B43" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="C43" s="44" t="s">
+      <c r="C43" s="8" t="s">
         <v>247</v>
       </c>
       <c r="D43" s="15" t="s">
@@ -15396,7 +15393,7 @@
       <c r="B44" s="8">
         <v>52</v>
       </c>
-      <c r="C44" s="44" t="s">
+      <c r="C44" s="8" t="s">
         <v>252</v>
       </c>
       <c r="D44" s="15" t="s">
@@ -15423,7 +15420,7 @@
       <c r="B45" s="8">
         <v>53</v>
       </c>
-      <c r="C45" s="44" t="s">
+      <c r="C45" s="8" t="s">
         <v>258</v>
       </c>
       <c r="D45" s="15" t="s">
@@ -15450,7 +15447,7 @@
       <c r="B46" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="C46" s="44" t="s">
+      <c r="C46" s="8" t="s">
         <v>265</v>
       </c>
       <c r="D46" s="15" t="s">
@@ -15477,7 +15474,7 @@
       <c r="B47" s="8">
         <v>54</v>
       </c>
-      <c r="C47" s="44" t="s">
+      <c r="C47" s="8" t="s">
         <v>270</v>
       </c>
       <c r="D47" s="15" t="s">
@@ -15504,7 +15501,7 @@
       <c r="B48" s="8">
         <v>55</v>
       </c>
-      <c r="C48" s="44" t="s">
+      <c r="C48" s="8" t="s">
         <v>275</v>
       </c>
       <c r="D48" s="15" t="s">
@@ -15531,7 +15528,7 @@
       <c r="B49" s="8" t="s">
         <v>281</v>
       </c>
-      <c r="C49" s="44" t="s">
+      <c r="C49" s="8" t="s">
         <v>282</v>
       </c>
       <c r="D49" s="15" t="s">
@@ -15558,7 +15555,7 @@
       <c r="B50" s="8">
         <v>60</v>
       </c>
-      <c r="C50" s="44" t="s">
+      <c r="C50" s="8" t="s">
         <v>287</v>
       </c>
       <c r="D50" s="15" t="s">
@@ -15585,7 +15582,7 @@
       <c r="B51" s="8">
         <v>62</v>
       </c>
-      <c r="C51" s="44" t="s">
+      <c r="C51" s="8" t="s">
         <v>292</v>
       </c>
       <c r="D51" s="15" t="s">
@@ -15612,7 +15609,7 @@
       <c r="B52" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="C52" s="44" t="s">
+      <c r="C52" s="8" t="s">
         <v>299</v>
       </c>
       <c r="D52" s="15" t="s">
@@ -15639,7 +15636,7 @@
       <c r="B53" s="8">
         <v>63</v>
       </c>
-      <c r="C53" s="44" t="s">
+      <c r="C53" s="8" t="s">
         <v>304</v>
       </c>
       <c r="D53" s="15" t="s">
@@ -15666,7 +15663,7 @@
       <c r="B54" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="C54" s="44" t="s">
+      <c r="C54" s="8" t="s">
         <v>310</v>
       </c>
       <c r="D54" s="15" t="s">
@@ -15693,7 +15690,7 @@
       <c r="B55" s="8">
         <v>64</v>
       </c>
-      <c r="C55" s="44" t="s">
+      <c r="C55" s="8" t="s">
         <v>315</v>
       </c>
       <c r="D55" s="15" t="s">
@@ -15720,7 +15717,7 @@
       <c r="B56" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="C56" s="44" t="s">
+      <c r="C56" s="8" t="s">
         <v>321</v>
       </c>
       <c r="D56" s="15" t="s">
@@ -15747,7 +15744,7 @@
       <c r="B57" s="8">
         <v>65</v>
       </c>
-      <c r="C57" s="44" t="s">
+      <c r="C57" s="8" t="s">
         <v>326</v>
       </c>
       <c r="D57" s="15" t="s">
@@ -15774,7 +15771,7 @@
       <c r="B58" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="C58" s="44" t="s">
+      <c r="C58" s="8" t="s">
         <v>332</v>
       </c>
       <c r="D58" s="15" t="s">
@@ -15801,7 +15798,7 @@
       <c r="B59" s="8">
         <v>66</v>
       </c>
-      <c r="C59" s="44" t="s">
+      <c r="C59" s="8" t="s">
         <v>337</v>
       </c>
       <c r="D59" s="15" t="s">
@@ -15828,7 +15825,7 @@
       <c r="B60" s="8">
         <v>67</v>
       </c>
-      <c r="C60" s="44" t="s">
+      <c r="C60" s="8" t="s">
         <v>342</v>
       </c>
       <c r="D60" s="15" t="s">
@@ -15855,7 +15852,7 @@
       <c r="B61" s="8">
         <v>68</v>
       </c>
-      <c r="C61" s="44" t="s">
+      <c r="C61" s="8" t="s">
         <v>347</v>
       </c>
       <c r="D61" s="15" t="s">
@@ -15882,7 +15879,7 @@
       <c r="B62" s="8">
         <v>69</v>
       </c>
-      <c r="C62" s="44" t="s">
+      <c r="C62" s="8" t="s">
         <v>352</v>
       </c>
       <c r="D62" s="15" t="s">
@@ -15909,7 +15906,7 @@
       <c r="B63" s="8" t="s">
         <v>358</v>
       </c>
-      <c r="C63" s="44" t="s">
+      <c r="C63" s="8" t="s">
         <v>359</v>
       </c>
       <c r="D63" s="15" t="s">
@@ -15936,7 +15933,7 @@
       <c r="B64" s="8">
         <v>70</v>
       </c>
-      <c r="C64" s="44" t="s">
+      <c r="C64" s="8" t="s">
         <v>364</v>
       </c>
       <c r="D64" s="14" t="s">
@@ -15963,7 +15960,7 @@
       <c r="B65" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="C65" s="44" t="s">
+      <c r="C65" s="8" t="s">
         <v>371</v>
       </c>
       <c r="D65" s="15" t="s">
@@ -15990,7 +15987,7 @@
       <c r="B66" s="8">
         <v>71</v>
       </c>
-      <c r="C66" s="44" t="s">
+      <c r="C66" s="8" t="s">
         <v>376</v>
       </c>
       <c r="D66" s="15" t="s">
@@ -16017,7 +16014,7 @@
       <c r="B67" s="8">
         <v>72</v>
       </c>
-      <c r="C67" s="44" t="s">
+      <c r="C67" s="8" t="s">
         <v>382</v>
       </c>
       <c r="D67" s="15" t="s">
@@ -16044,7 +16041,7 @@
       <c r="B68" s="8" t="s">
         <v>388</v>
       </c>
-      <c r="C68" s="44" t="s">
+      <c r="C68" s="8" t="s">
         <v>389</v>
       </c>
       <c r="D68" s="15" t="s">
@@ -16071,7 +16068,7 @@
       <c r="B69" s="8">
         <v>73</v>
       </c>
-      <c r="C69" s="44" t="s">
+      <c r="C69" s="8" t="s">
         <v>394</v>
       </c>
       <c r="D69" s="15" t="s">
@@ -16098,7 +16095,7 @@
       <c r="B70" s="8">
         <v>74</v>
       </c>
-      <c r="C70" s="44" t="s">
+      <c r="C70" s="8" t="s">
         <v>399</v>
       </c>
       <c r="D70" s="15" t="s">
@@ -16125,7 +16122,7 @@
       <c r="B71" s="8">
         <v>75</v>
       </c>
-      <c r="C71" s="44" t="s">
+      <c r="C71" s="8" t="s">
         <v>404</v>
       </c>
       <c r="D71" s="15" t="s">
@@ -16152,7 +16149,7 @@
       <c r="B72" s="8">
         <v>76</v>
       </c>
-      <c r="C72" s="44" t="s">
+      <c r="C72" s="8" t="s">
         <v>409</v>
       </c>
       <c r="D72" s="14" t="s">
@@ -16179,7 +16176,7 @@
       <c r="B73" s="8">
         <v>77</v>
       </c>
-      <c r="C73" s="44" t="s">
+      <c r="C73" s="8" t="s">
         <v>414</v>
       </c>
       <c r="D73" s="15" t="s">
@@ -16206,7 +16203,7 @@
       <c r="B74" s="8">
         <v>78</v>
       </c>
-      <c r="C74" s="44" t="s">
+      <c r="C74" s="8" t="s">
         <v>420</v>
       </c>
       <c r="D74" s="15" t="s">
@@ -16233,7 +16230,7 @@
       <c r="B75" s="8">
         <v>79</v>
       </c>
-      <c r="C75" s="44" t="s">
+      <c r="C75" s="8" t="s">
         <v>425</v>
       </c>
       <c r="D75" s="15" t="s">
@@ -16260,7 +16257,7 @@
       <c r="B76" s="8">
         <v>246</v>
       </c>
-      <c r="C76" s="44" t="s">
+      <c r="C76" s="8" t="s">
         <v>430</v>
       </c>
       <c r="D76" s="15" t="s">
@@ -16287,7 +16284,7 @@
       <c r="B77" s="8">
         <v>247</v>
       </c>
-      <c r="C77" s="44" t="s">
+      <c r="C77" s="8" t="s">
         <v>435</v>
       </c>
       <c r="D77" s="15" t="s">
@@ -16314,7 +16311,7 @@
       <c r="B78" s="8">
         <v>248</v>
       </c>
-      <c r="C78" s="44" t="s">
+      <c r="C78" s="8" t="s">
         <v>440</v>
       </c>
       <c r="D78" s="15" t="s">
@@ -16341,7 +16338,7 @@
       <c r="B79" s="8" t="s">
         <v>445</v>
       </c>
-      <c r="C79" s="44" t="s">
+      <c r="C79" s="8" t="s">
         <v>446</v>
       </c>
       <c r="D79" s="15" t="s">
@@ -16368,7 +16365,7 @@
       <c r="B80" s="8">
         <v>249</v>
       </c>
-      <c r="C80" s="44" t="s">
+      <c r="C80" s="8" t="s">
         <v>451</v>
       </c>
       <c r="D80" s="15" t="s">
@@ -16395,7 +16392,7 @@
       <c r="B81" s="8" t="s">
         <v>456</v>
       </c>
-      <c r="C81" s="44" t="s">
+      <c r="C81" s="8" t="s">
         <v>457</v>
       </c>
       <c r="D81" s="15" t="s">
@@ -16422,7 +16419,7 @@
       <c r="B82" s="8">
         <v>250</v>
       </c>
-      <c r="C82" s="44" t="s">
+      <c r="C82" s="8" t="s">
         <v>462</v>
       </c>
       <c r="D82" s="14" t="s">
@@ -16451,7 +16448,7 @@
       <c r="B83" s="8">
         <v>253</v>
       </c>
-      <c r="C83" s="44" t="s">
+      <c r="C83" s="8" t="s">
         <v>467</v>
       </c>
       <c r="D83" s="15" t="s">
@@ -16480,7 +16477,7 @@
       <c r="B84" s="8" t="s">
         <v>472</v>
       </c>
-      <c r="C84" s="44" t="s">
+      <c r="C84" s="8" t="s">
         <v>473</v>
       </c>
       <c r="D84" s="15" t="s">
@@ -16509,7 +16506,7 @@
       <c r="B85" s="8">
         <v>254</v>
       </c>
-      <c r="C85" s="44" t="s">
+      <c r="C85" s="8" t="s">
         <v>478</v>
       </c>
       <c r="D85" s="15" t="s">
@@ -16538,7 +16535,7 @@
       <c r="B86" s="8" t="s">
         <v>483</v>
       </c>
-      <c r="C86" s="44" t="s">
+      <c r="C86" s="8" t="s">
         <v>484</v>
       </c>
       <c r="D86" s="15" t="s">
@@ -16567,7 +16564,7 @@
       <c r="B87" s="8">
         <v>256</v>
       </c>
-      <c r="C87" s="44" t="s">
+      <c r="C87" s="8" t="s">
         <v>489</v>
       </c>
       <c r="D87" s="15" t="s">
@@ -16596,7 +16593,7 @@
       <c r="B88" s="8">
         <v>257</v>
       </c>
-      <c r="C88" s="44" t="s">
+      <c r="C88" s="8" t="s">
         <v>494</v>
       </c>
       <c r="D88" s="15" t="s">
@@ -16625,7 +16622,7 @@
       <c r="B89" s="8">
         <v>258</v>
       </c>
-      <c r="C89" s="44" t="s">
+      <c r="C89" s="8" t="s">
         <v>499</v>
       </c>
       <c r="D89" s="15" t="s">
@@ -16654,7 +16651,7 @@
       <c r="B90" s="8">
         <v>259</v>
       </c>
-      <c r="C90" s="44" t="s">
+      <c r="C90" s="8" t="s">
         <v>504</v>
       </c>
       <c r="D90" s="15" t="s">
@@ -16683,7 +16680,7 @@
       <c r="B91" s="8">
         <v>260</v>
       </c>
-      <c r="C91" s="44" t="s">
+      <c r="C91" s="8" t="s">
         <v>509</v>
       </c>
       <c r="D91" s="15" t="s">
@@ -16712,7 +16709,7 @@
       <c r="B92" s="8">
         <v>261</v>
       </c>
-      <c r="C92" s="44" t="s">
+      <c r="C92" s="8" t="s">
         <v>514</v>
       </c>
       <c r="D92" s="15" t="s">
@@ -16741,7 +16738,7 @@
       <c r="B93" s="8">
         <v>262</v>
       </c>
-      <c r="C93" s="44" t="s">
+      <c r="C93" s="8" t="s">
         <v>519</v>
       </c>
       <c r="D93" s="14" t="s">
@@ -16771,7 +16768,7 @@
       <c r="B94" s="8">
         <v>263</v>
       </c>
-      <c r="C94" s="44" t="s">
+      <c r="C94" s="8" t="s">
         <v>524</v>
       </c>
       <c r="D94" s="15" t="s">
@@ -16801,7 +16798,7 @@
       <c r="B95" s="8">
         <v>264</v>
       </c>
-      <c r="C95" s="44" t="s">
+      <c r="C95" s="8" t="s">
         <v>529</v>
       </c>
       <c r="D95" s="15" t="s">
@@ -16831,7 +16828,7 @@
       <c r="B96" s="8" t="s">
         <v>534</v>
       </c>
-      <c r="C96" s="44" t="s">
+      <c r="C96" s="8" t="s">
         <v>535</v>
       </c>
       <c r="D96" s="15" t="s">
@@ -16861,7 +16858,7 @@
       <c r="B97" s="8">
         <v>265</v>
       </c>
-      <c r="C97" s="44" t="s">
+      <c r="C97" s="8" t="s">
         <v>540</v>
       </c>
       <c r="D97" s="15" t="s">
@@ -16891,7 +16888,7 @@
       <c r="B98" s="8">
         <v>266</v>
       </c>
-      <c r="C98" s="44" t="s">
+      <c r="C98" s="8" t="s">
         <v>545</v>
       </c>
       <c r="D98" s="15" t="s">
@@ -16921,7 +16918,7 @@
       <c r="B99" s="8">
         <v>267</v>
       </c>
-      <c r="C99" s="44" t="s">
+      <c r="C99" s="8" t="s">
         <v>550</v>
       </c>
       <c r="D99" s="15" t="s">
@@ -16951,7 +16948,7 @@
       <c r="B100" s="8">
         <v>268</v>
       </c>
-      <c r="C100" s="44" t="s">
+      <c r="C100" s="8" t="s">
         <v>555</v>
       </c>
       <c r="D100" s="15" t="s">
@@ -16981,7 +16978,7 @@
       <c r="B101" s="8">
         <v>269</v>
       </c>
-      <c r="C101" s="44" t="s">
+      <c r="C101" s="8" t="s">
         <v>560</v>
       </c>
       <c r="D101" s="14" t="s">
@@ -17011,7 +17008,7 @@
       <c r="B102" s="8">
         <v>270</v>
       </c>
-      <c r="C102" s="44" t="s">
+      <c r="C102" s="8" t="s">
         <v>565</v>
       </c>
       <c r="D102" s="15" t="s">
@@ -17041,7 +17038,7 @@
       <c r="B103" s="8">
         <v>271</v>
       </c>
-      <c r="C103" s="44" t="s">
+      <c r="C103" s="8" t="s">
         <v>570</v>
       </c>
       <c r="D103" s="15" t="s">
@@ -17071,7 +17068,7 @@
       <c r="B104" s="8">
         <v>272</v>
       </c>
-      <c r="C104" s="44" t="s">
+      <c r="C104" s="8" t="s">
         <v>576</v>
       </c>
       <c r="D104" s="15" t="s">
@@ -17101,7 +17098,7 @@
       <c r="B105" s="8">
         <v>273</v>
       </c>
-      <c r="C105" s="44" t="s">
+      <c r="C105" s="8" t="s">
         <v>581</v>
       </c>
       <c r="D105" s="20" t="s">
@@ -17131,7 +17128,7 @@
       <c r="B106" s="8">
         <v>274</v>
       </c>
-      <c r="C106" s="44" t="s">
+      <c r="C106" s="8" t="s">
         <v>586</v>
       </c>
       <c r="D106" s="20" t="s">
@@ -17163,7 +17160,7 @@
       <c r="B107" s="8">
         <v>275</v>
       </c>
-      <c r="C107" s="44" t="s">
+      <c r="C107" s="8" t="s">
         <v>591</v>
       </c>
       <c r="D107" s="20" t="s">
@@ -17194,7 +17191,7 @@
       <c r="B108" s="8">
         <v>276</v>
       </c>
-      <c r="C108" s="44" t="s">
+      <c r="C108" s="8" t="s">
         <v>596</v>
       </c>
       <c r="D108" s="22" t="s">
@@ -17224,7 +17221,7 @@
       <c r="B109" s="8">
         <v>277</v>
       </c>
-      <c r="C109" s="44" t="s">
+      <c r="C109" s="8" t="s">
         <v>601</v>
       </c>
       <c r="D109" s="22" t="s">
@@ -17254,7 +17251,7 @@
       <c r="B110" s="8">
         <v>278</v>
       </c>
-      <c r="C110" s="44" t="s">
+      <c r="C110" s="8" t="s">
         <v>606</v>
       </c>
       <c r="D110" s="22" t="s">
@@ -17284,7 +17281,7 @@
       <c r="B111" s="8">
         <v>283</v>
       </c>
-      <c r="C111" s="44" t="s">
+      <c r="C111" s="8" t="s">
         <v>611</v>
       </c>
       <c r="D111" s="22" t="s">
@@ -17314,7 +17311,7 @@
       <c r="B112" s="8">
         <v>284</v>
       </c>
-      <c r="C112" s="44" t="s">
+      <c r="C112" s="8" t="s">
         <v>616</v>
       </c>
       <c r="D112" s="22" t="s">
@@ -17344,7 +17341,7 @@
       <c r="B113" s="8" t="s">
         <v>621</v>
       </c>
-      <c r="C113" s="44" t="s">
+      <c r="C113" s="8" t="s">
         <v>622</v>
       </c>
       <c r="D113" s="20" t="s">
@@ -17374,7 +17371,7 @@
       <c r="B114" s="8">
         <v>285</v>
       </c>
-      <c r="C114" s="44" t="s">
+      <c r="C114" s="8" t="s">
         <v>627</v>
       </c>
       <c r="D114" s="15" t="s">
@@ -17404,7 +17401,7 @@
       <c r="B115" s="8">
         <v>286</v>
       </c>
-      <c r="C115" s="44" t="s">
+      <c r="C115" s="8" t="s">
         <v>633</v>
       </c>
       <c r="D115" s="15" t="s">
@@ -17434,7 +17431,7 @@
       <c r="B116" s="8">
         <v>287</v>
       </c>
-      <c r="C116" s="44" t="s">
+      <c r="C116" s="8" t="s">
         <v>638</v>
       </c>
       <c r="D116" s="15" t="s">
@@ -17464,7 +17461,7 @@
       <c r="B117" s="8">
         <v>288</v>
       </c>
-      <c r="C117" s="44" t="s">
+      <c r="C117" s="8" t="s">
         <v>643</v>
       </c>
       <c r="D117" s="15" t="s">
@@ -17494,7 +17491,7 @@
       <c r="B118" s="8">
         <v>289</v>
       </c>
-      <c r="C118" s="44" t="s">
+      <c r="C118" s="8" t="s">
         <v>648</v>
       </c>
       <c r="D118" s="15" t="s">
@@ -17524,7 +17521,7 @@
       <c r="B119" s="8">
         <v>290</v>
       </c>
-      <c r="C119" s="44" t="s">
+      <c r="C119" s="8" t="s">
         <v>653</v>
       </c>
       <c r="D119" s="15" t="s">
@@ -17554,7 +17551,7 @@
       <c r="B120" s="8">
         <v>291</v>
       </c>
-      <c r="C120" s="44" t="s">
+      <c r="C120" s="8" t="s">
         <v>659</v>
       </c>
       <c r="D120" s="6" t="s">
@@ -17581,7 +17578,7 @@
       <c r="B121" s="8">
         <v>292</v>
       </c>
-      <c r="C121" s="44" t="s">
+      <c r="C121" s="8" t="s">
         <v>664</v>
       </c>
       <c r="D121" s="6" t="s">
@@ -17608,7 +17605,7 @@
       <c r="B122" s="8">
         <v>293</v>
       </c>
-      <c r="C122" s="44" t="s">
+      <c r="C122" s="8" t="s">
         <v>669</v>
       </c>
       <c r="D122" s="6" t="s">
@@ -17635,7 +17632,7 @@
       <c r="B123" s="8">
         <v>294</v>
       </c>
-      <c r="C123" s="44" t="s">
+      <c r="C123" s="8" t="s">
         <v>674</v>
       </c>
       <c r="D123" s="6" t="s">
@@ -17662,7 +17659,7 @@
       <c r="B124" s="8" t="s">
         <v>680</v>
       </c>
-      <c r="C124" s="44" t="s">
+      <c r="C124" s="8" t="s">
         <v>681</v>
       </c>
       <c r="D124" s="6" t="s">
@@ -17689,7 +17686,7 @@
       <c r="B125" s="8">
         <v>296</v>
       </c>
-      <c r="C125" s="44" t="s">
+      <c r="C125" s="8" t="s">
         <v>686</v>
       </c>
       <c r="D125" s="6" t="s">
@@ -17716,7 +17713,7 @@
       <c r="B126" s="8">
         <v>298</v>
       </c>
-      <c r="C126" s="44" t="s">
+      <c r="C126" s="8" t="s">
         <v>691</v>
       </c>
       <c r="D126" s="6" t="s">

</xml_diff>